<commit_message>
Update Task 1 data
</commit_message>
<xml_diff>
--- a/Task1.xlsx
+++ b/Task1.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="6" documentId="11_74955360D2368D840378C7DA176E042778FBF945" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E760E1BD-7E71-4470-BB3C-F19DDE646258}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="11_74955360D2368D840378C7DA176E042778FBF945" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{98161149-769B-4E9D-B4AF-AF33748D11F0}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="179">
   <si>
     <t>Name</t>
   </si>
@@ -549,6 +549,12 @@
   </si>
   <si>
     <t>John Kennedy Avenue, Curepipe</t>
+  </si>
+  <si>
+    <t>16, Maxime Rémi Street, Camp Le Vieux, Roches Brunes</t>
+  </si>
+  <si>
+    <t>Royal Road , Beau Bassin - Rose Hill</t>
   </si>
 </sst>
 </file>
@@ -1221,6 +1227,9 @@
       <c r="B18" t="s">
         <v>7</v>
       </c>
+      <c r="C18" t="s">
+        <v>178</v>
+      </c>
       <c r="D18" t="s">
         <v>44</v>
       </c>
@@ -1278,6 +1287,9 @@
       <c r="B21" t="s">
         <v>7</v>
       </c>
+      <c r="C21" t="s">
+        <v>177</v>
+      </c>
       <c r="D21" t="s">
         <v>57</v>
       </c>
@@ -1345,6 +1357,9 @@
       </c>
       <c r="B25" t="s">
         <v>7</v>
+      </c>
+      <c r="C25" t="s">
+        <v>105</v>
       </c>
       <c r="D25" t="s">
         <v>66</v>

</xml_diff>